<commit_message>
checkpoint: aggregate cross-dataset pipeline + MBRT-vs-SBRT analysis plan
Captures the working-tree state at the aggregate-typing lock and the
downstream differential-analysis design:

- aggregate.smk + scripts/aggregate/* tier-1/2 cross-dataset typing
  (scVI integration, Leiden cluster-then-annotate, SingleR/UCell
  subtyping with marker-rescue) and its result tables/figures
- plan-mbrt-vs-sbrt.md (approved design spec) + plan-mbrt-vs-sbrt-impl.md
  (implementation plan, to be executed in a new session); indexed from
  the org notebook Plans heading
- config/lineage_markers.yaml, config/spatial-rads-scvi-env.yaml
- dev/ exploratory work (mbrt_vs_sbrt, if_channel_check, peak/valley
  signatures) retained as method provenance, not pipeline code
- metadata cleanup: drop root metadata.xlsx + duplicate panel XLSX
  (canonical copy lives in data/)
- .gitignore: exclude heavy regenerable binaries (rds/parquet/tsv.gz/
  pptx), large aggregate dumps, run artifacts, and local .claude/ settings
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -11,6 +11,7 @@
     <sheet name="datasets" sheetId="2" r:id="rId2"/>
     <sheet name="slides" sheetId="3" r:id="rId3"/>
     <sheet name="samples" sheetId="4" r:id="rId4"/>
+    <sheet name="if_channels" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -662,7 +663,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -688,20 +689,45 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>panel_base</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>panel_custom</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>assay_type</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>n_negprobe</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>n_falsecode</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>provider</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>format</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>counts_path</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>metadata_path</t>
         </is>
@@ -728,20 +754,35 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Mouse UCC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Alan Fields 21-gene</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>RNA</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Yi Liu / Mutter Lab</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>parquet</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>/mnt/data/projects/spatial-rads/inputs/mutter01/projects_Mutter_01_CosMmR_app_data_raw_tx_counts_matrix.parquet</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>/mnt/data/projects/spatial-rads/inputs/mutter01/Analysis_Mutter_01_CosMmR_Mutter_updated_metadata.parquet</t>
         </is>
@@ -768,10 +809,31 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>Mouse UCC</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1K_Mayo_Thomp-Fields1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>RNA</t>
+        </is>
+      </c>
+      <c r="H3">
+        <v>10</v>
+      </c>
+      <c r="I3">
+        <v>184</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>Mutter Lab</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>rds</t>
         </is>
@@ -2329,4 +2391,326 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>meta_cols</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dat0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CD298.B2M</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>B2M/CD298</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>segmentation_membrane</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mean.CD298.B2M;Max.CD298.B2M</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dat0001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CD45</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PTPRC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>lineage_immune</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mean.CD45;Max.CD45</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dat0001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DAPI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DNA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>segmentation_nuclear</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mean.DAPI;Max.DAPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dat0001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>unspecified</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>redundant_epithelial</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mean.G;Max.G</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>r~0.92 with Mean.PanCK; not a literal duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dat0001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PanCK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pan-cytokeratin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>lineage_epithelial</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mean.PanCK;Max.PanCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dat0002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CD298.B2M</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B2M/CD298</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>segmentation_membrane</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Mean.CD298.B2M;Max.CD298.B2M</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dat0002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CD45</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PTPRC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>lineage_immune</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Mean.CD45;Max.CD45</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dat0002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DAPI</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DNA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>segmentation_nuclear</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Mean.DAPI;Max.DAPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dat0002</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>unspecified</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>redundant_epithelial</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Mean.G;Max.G</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>r~0.92 with Mean.PanCK; not a literal duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dat0002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PanCK</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>pan-cytokeratin</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>lineage_epithelial</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mean.PanCK;Max.PanCK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(processing): contamination QC (MECR) + M01 raw-RDS adapter re-base
Report-only contamination_qc rule (SpatialQM MECR, per-sample + per-FOV with
necrosis / mixed-biology triage columns; FastReseg infeasible). adapt_mutter01
re-based onto the 4 per-slide RDS (counts byte-identical to the parquet, invariance
verified); data model flipped to format=rds. Org-tangled; processing.smk dry-run clean.

Claude-Session: https://claude.ai/code/session_012uKDWF2ExcwbqkD5mcsFtn
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -767,6 +767,12 @@
           <t>RNA</t>
         </is>
       </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+      <c r="I2">
+        <v>184</v>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>Yi Liu / Mutter Lab</t>
@@ -774,12 +780,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>parquet</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>/mnt/data/projects/spatial-rads/inputs/mutter01/projects_Mutter_01_CosMmR_app_data_raw_tx_counts_matrix.parquet</t>
+          <t>rds</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -887,6 +888,11 @@
           <t>20250529_214712_S1</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>/mnt/data/projects/spatial-rads/inputs/mutter01/seuratObject_01_Mutter_01_CosMmR.RDS</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -904,6 +910,11 @@
           <t>20250529_214712_S2</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>/mnt/data/projects/spatial-rads/inputs/mutter01/seuratObject_02_Mutter_01_CosMmR.RDS</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -921,6 +932,11 @@
           <t>20250529_214712_S3</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>/mnt/data/projects/spatial-rads/inputs/mutter01/seuratObject_03_Mutter_01_CosMmR.RDS</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -936,6 +952,11 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>20250529_214712_S4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>/mnt/data/projects/spatial-rads/inputs/mutter01/seuratObject_04_Mutter_01_CosMmR.RDS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(m02): apply M02 timepoint relabel, per-cell_type BH, stroma rename, plan cleanup
M02 slides 3-4 are 4h (not day-2): metadata, comparisons registry, and
engine cohort whitelist corrected. Arm table padj switched from pooled BH
to per-cell_type BH (field-standard per Crowell et al. 2020 muscat).
"unassigned" stroma renamed to "stroma_unresolved" in typing scripts and
docs. Producer scripts generalized from M02-only to all-flank. Completed
plans removed (rotation-null, differential-robustness, mbrt-vs-sbrt,
aggregate-refactor, svg-v2).

Claude-Session: https://claude.ai/code/session_01MTxDsUXqHQEpgYtBT7vTde
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MBRT_day2</t>
+          <t>MBRT_4h</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="H20">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SBRT_day2</t>
+          <t>SBRT_4h</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2215,7 +2215,7 @@
         <v>20</v>
       </c>
       <c r="H21">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MBRT_day2</t>
+          <t>MBRT_4h</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2328,7 +2328,7 @@
         </is>
       </c>
       <c r="H23">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SBRT_day2</t>
+          <t>SBRT_4h</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2386,7 +2386,7 @@
         <v>20</v>
       </c>
       <c r="H24">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>

</xml_diff>